<commit_message>
T-shirts : 13 mises en page uniques + illustrations Canva (pilote), lot 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017s9aiUQGwXkQS3gVkKXYXa
</commit_message>
<xml_diff>
--- a/tshirts/banque-slogans.xlsx
+++ b/tshirts/banque-slogans.xlsx
@@ -1186,7 +1186,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Design fait</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Site boutique : pages, paiement Stripe, commande Printful, publication, choix du t-shirt et prix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017s9aiUQGwXkQS3gVkKXYXa
</commit_message>
<xml_diff>
--- a/tshirts/banque-slogans.xlsx
+++ b/tshirts/banque-slogans.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Slogans'!$A$1:$H$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Slogans'!$A$1:$J$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -86,7 +86,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -119,6 +119,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFD8A8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -484,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -495,6 +502,8 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,6 +547,16 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Style choisi</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>ID design</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -578,6 +597,16 @@
           <t>Design déjà généré</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>plaque</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>petanque-apero</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -618,6 +647,16 @@
           <t>Design déjà généré</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>coucher</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>camping-car</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -654,6 +693,16 @@
           <t>Design déjà généré</t>
         </is>
       </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>graines</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>jardin-tomates</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -694,6 +743,16 @@
           <t>Design déjà généré</t>
         </is>
       </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>tampon</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>caractere</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -734,6 +793,16 @@
           <t>Design déjà généré</t>
         </is>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>diplome</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>retraite</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -774,6 +843,12 @@
           <t>Style fiche</t>
         </is>
       </c>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>mode-papy</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -810,6 +885,8 @@
           <t>TON IDÉE. Risque : PureTech est une marque déposée de Stellantis. Préférer la version sans nom ci-dessous.</t>
         </is>
       </c>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -850,6 +927,12 @@
           <t>Version sans marque : les mécanos comprennent tout de suite</t>
         </is>
       </c>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>mecano-courroie</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -886,6 +969,12 @@
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>mecano-tuto</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -922,6 +1011,16 @@
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>ticket</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>beau-frere-repare</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -954,6 +1053,12 @@
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>mecano-ecologie</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -990,6 +1095,16 @@
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>bd</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>mecano-oreille</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1022,6 +1137,16 @@
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>recherche</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>plombier-davant</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1054,6 +1179,12 @@
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>plombier-fuite</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1090,6 +1221,12 @@
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>plombier-secrets</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1126,6 +1263,16 @@
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>dico</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>electricien-domino</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1158,6 +1305,12 @@
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>electricien-1998</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1190,6 +1343,12 @@
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>electricien-tension</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1226,6 +1385,16 @@
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>chantier</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>macon-enduit</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1258,6 +1427,12 @@
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>plaquiste-ba13</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1290,6 +1465,12 @@
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>devis-juste</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1322,6 +1503,12 @@
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>chantier-vendredi</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1358,6 +1545,12 @@
           <t>Ton terrain : idéal pour tester</t>
         </is>
       </c>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>couvreur-flemme</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1390,6 +1583,16 @@
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>couvreur-pigeons</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1426,6 +1629,12 @@
           <t>13,60 m = longueur d'une remorque standard</t>
         </is>
       </c>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>routier-1360</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1458,6 +1667,16 @@
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>panneau</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>routier-rondspoints</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1490,6 +1709,12 @@
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>agriculteur-70h</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1526,6 +1751,8 @@
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1558,6 +1785,8 @@
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1594,6 +1823,8 @@
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1626,6 +1857,8 @@
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1658,6 +1891,8 @@
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1690,6 +1925,8 @@
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1726,6 +1963,8 @@
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1758,6 +1997,8 @@
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1790,6 +2031,8 @@
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1822,6 +2065,8 @@
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1854,6 +2099,8 @@
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1886,6 +2133,8 @@
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1918,6 +2167,8 @@
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1950,6 +2201,8 @@
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1982,6 +2235,8 @@
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2014,6 +2269,8 @@
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2046,6 +2303,8 @@
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2078,6 +2337,8 @@
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2110,6 +2371,8 @@
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2146,6 +2409,8 @@
           <t>Un peu limite</t>
         </is>
       </c>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2182,6 +2447,8 @@
           <t>Un peu limite · blague connue, à tester</t>
         </is>
       </c>
+      <c r="I49" s="2" t="n"/>
+      <c r="J49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2218,6 +2485,8 @@
           <t>Un peu limite</t>
         </is>
       </c>
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2254,6 +2523,8 @@
           <t>Un peu limite</t>
         </is>
       </c>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2290,6 +2561,16 @@
           <t>Un peu limite</t>
         </is>
       </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>etiquette</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>saucisson-aux-herbes</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2322,6 +2603,8 @@
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2358,6 +2641,8 @@
           <t>Autodérision : OK car il parle de lui</t>
         </is>
       </c>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2394,6 +2679,8 @@
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2430,6 +2717,8 @@
           <t>Un peu limite · pub Meta parfois refusée sur l'alcool</t>
         </is>
       </c>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2466,6 +2755,8 @@
           <t>Pub Meta parfois refusée sur l'alcool</t>
         </is>
       </c>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2502,6 +2793,8 @@
           <t>Un peu limite · fait réagir en commentaires</t>
         </is>
       </c>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2538,6 +2831,8 @@
           <t>Marche très bien en province</t>
         </is>
       </c>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -2574,6 +2869,8 @@
           <t>À décliner par région</t>
         </is>
       </c>
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2606,6 +2903,8 @@
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2638,6 +2937,8 @@
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -2670,6 +2971,8 @@
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2702,6 +3005,8 @@
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -2734,6 +3039,8 @@
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -2766,6 +3073,8 @@
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2798,6 +3107,8 @@
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2834,6 +3145,8 @@
           <t>TON IDÉE. Illustration obligatoire (verre de pastis + verre de rouge) pour que le double sens soit compris en 1 seconde. Risque de signalements si lu au premier degré.</t>
         </is>
       </c>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -2874,6 +3187,8 @@
           <t>Variante plus sûre de ton idée : le rosé rend le sens évident</t>
         </is>
       </c>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -2910,6 +3225,8 @@
           <t>Illustration : verre de vin + feuille de salade</t>
         </is>
       </c>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -2946,6 +3263,8 @@
           <t>Cible femme, été</t>
         </is>
       </c>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -2982,6 +3301,8 @@
           <t>Illustration : poche de sang façon bouteille</t>
         </is>
       </c>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3014,6 +3335,8 @@
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="n"/>
+      <c r="J73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3050,6 +3373,8 @@
           <t>Illustration : verre de pastis avec paille et parasol</t>
         </is>
       </c>
+      <c r="I74" s="2" t="n"/>
+      <c r="J74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3086,6 +3411,8 @@
           <t>Illustration : bonhomme en tire-bouchon</t>
         </is>
       </c>
+      <c r="I75" s="2" t="n"/>
+      <c r="J75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3118,6 +3445,8 @@
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="n"/>
+      <c r="J76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3150,6 +3479,8 @@
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="n"/>
+      <c r="J77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3186,6 +3517,8 @@
           <t>Très bon cadeau anniversaire 50/60 ans</t>
         </is>
       </c>
+      <c r="I78" s="2" t="n"/>
+      <c r="J78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3222,6 +3555,8 @@
           <t>Cible retraités</t>
         </is>
       </c>
+      <c r="I79" s="2" t="n"/>
+      <c r="J79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3258,6 +3593,8 @@
           <t>Tomate = pastis grenadine. Illustration : verre de pastis rouge avec une feuille de tomate</t>
         </is>
       </c>
+      <c r="I80" s="2" t="n"/>
+      <c r="J80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -3294,6 +3631,8 @@
           <t>Momie = petite dose. Illustration : verre de pastis avec bandelettes et couronne de pharaon</t>
         </is>
       </c>
+      <c r="I81" s="2" t="n"/>
+      <c r="J81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -3330,6 +3669,8 @@
           <t>Les initiés comprennent tout de suite</t>
         </is>
       </c>
+      <c r="I82" s="2" t="n"/>
+      <c r="J82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -3362,6 +3703,8 @@
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="n"/>
+      <c r="J83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -3402,6 +3745,8 @@
           <t>Illustration : feu tricolore avec un verre de pastis à la place de l'orange</t>
         </is>
       </c>
+      <c r="I84" s="2" t="n"/>
+      <c r="J84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -3438,6 +3783,8 @@
           <t>Débat de comptoir qui fait commenter</t>
         </is>
       </c>
+      <c r="I85" s="2" t="n"/>
+      <c r="J85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -3470,6 +3817,8 @@
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="n"/>
+      <c r="J86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -3506,6 +3855,8 @@
           <t>Illustration : verre de whisky avec deux glaçons qui se tournent le dos</t>
         </is>
       </c>
+      <c r="I87" s="2" t="n"/>
+      <c r="J87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -3538,6 +3889,8 @@
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="n"/>
+      <c r="J88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -3574,6 +3927,8 @@
           <t>Daron vénère, très court = très lisible</t>
         </is>
       </c>
+      <c r="I89" s="2" t="n"/>
+      <c r="J89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -3606,6 +3961,8 @@
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="n"/>
+      <c r="J90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -3642,6 +3999,8 @@
           <t>Illustration : ballon de foot transformé en verre de vin</t>
         </is>
       </c>
+      <c r="I91" s="2" t="n"/>
+      <c r="J91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -3678,6 +4037,8 @@
           <t>Illustration : cubi souriant</t>
         </is>
       </c>
+      <c r="I92" s="2" t="n"/>
+      <c r="J92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -3718,6 +4079,8 @@
           <t>Court et efficace</t>
         </is>
       </c>
+      <c r="I93" s="2" t="n"/>
+      <c r="J93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -3750,6 +4113,8 @@
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="n"/>
+      <c r="J94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -3782,6 +4147,8 @@
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="n"/>
+      <c r="J95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -3818,6 +4185,8 @@
           <t>Illustration : pinte avec des jumelles</t>
         </is>
       </c>
+      <c r="I96" s="2" t="n"/>
+      <c r="J96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -3854,6 +4223,8 @@
           <t>Illustration : fût de bière en coupe</t>
         </is>
       </c>
+      <c r="I97" s="2" t="n"/>
+      <c r="J97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -3886,6 +4257,8 @@
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="n"/>
+      <c r="J98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -3922,6 +4295,8 @@
           <t>Illustration : pomme avec un bouchon de bouteille</t>
         </is>
       </c>
+      <c r="I99" s="2" t="n"/>
+      <c r="J99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -3958,6 +4333,8 @@
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="n"/>
+      <c r="J100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -3994,6 +4371,8 @@
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="n"/>
+      <c r="J101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -4030,6 +4409,8 @@
           <t>Référence aux campagnes Sécurité routière : tout le monde comprend. Positif (il ne conduit pas)</t>
         </is>
       </c>
+      <c r="I102" s="2" t="n"/>
+      <c r="J102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -4062,6 +4443,8 @@
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="n"/>
+      <c r="J103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -4094,9 +4477,241 @@
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="n"/>
+      <c r="J104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Vacances / caravane</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Ma maison a des roues et mon jardin change tous les jours (hérisson en chaise longue)</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr"/>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Mixte</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Design fait</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Style visuel + illustration Canva</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>visuel</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>caravane-herisson</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Vacances / caravane</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Ma maison a des roues et mon jardin change tous les jours (hérisson jardinier)</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr"/>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Mixte</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Design fait</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Style visuel + illustration Canva</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>visuel</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>caravane-herisson-jardin</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Régions – Corse</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>En Corse on est très accueillants… mais si tu klaxonnes dans un virage, tu repars à la nage</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr"/>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Mixte</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Design fait</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Style visuel + illustration Canva</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>visuel</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>corse-klaxon</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Régions – Corse</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>On est hyper accueillants. C'est juste qu'on préfère quand vous repartez.</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr"/>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Mixte</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Design fait</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Style visuel + illustration Canva</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>visuel</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>corse-repartez</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Régions – Corse</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>En Corse on est très accueillants… mais garde tes tongs pour la plage, pas pour le GR20</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr"/>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Mixte</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Design fait</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Style visuel + illustration Canva</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>visuel</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>corse-gr20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H104"/>
+  <autoFilter ref="A1:J109"/>
   <conditionalFormatting sqref="A2:H1000">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$G2="Validé"</formula>
@@ -4114,7 +4729,12 @@
       <formula>$G2="Abandonné"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <conditionalFormatting sqref="A2:J1000">
+    <cfRule type="expression" priority="6" dxfId="5">
+      <formula>$G2="À publier"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"noir,blanc,kaki,marine,sable,gris"</formula1>
     </dataValidation>
@@ -4122,7 +4742,10 @@
       <formula1>"H,F,Mixte"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Idée,Validé,Design fait,En ligne,Vendu,Abandonné,Test"</formula1>
+      <formula1>"Idée,Validé,Design fait,À publier,En aperçu,En ligne,Vendu,Abandonné,Test"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"visuel,empile,mix,badge,retro,fiche,illustre,etiquette,coucher,recherche,panneau,bd,graines,tampon,diplome,college,plaque,dico,ticket,chantier"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4358,7 +4981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -4399,6 +5022,13 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>6. Pour mettre un t-shirt en vente : choisis son style (colonne « Style choisi »), mets le statut « À publier », puis tape /publier.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>